<commit_message>
Add recommendation tabs to lead analysis workbook
Adds three tabs after Source Summary: Recommendation Summary (channel
ranking by cost-per-sold-estimate + guardrails), Budget Options (three
monthly budget scenarios), and Action Plan (no-cost fixes + 90-day
rollout) — mirroring the recommendation memo inside the spreadsheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YQamPWmLKgVpu8941r9uc9
</commit_message>
<xml_diff>
--- a/charlotte_lead_analysis/PatchitUP_Charlotte_Lead_Analysis.xlsx
+++ b/charlotte_lead_analysis/PatchitUP_Charlotte_Lead_Analysis.xlsx
@@ -8,8 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Source Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lead-Level Match" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GHL All Sources (Booked)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Recommendation Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Budget Options" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Action Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lead-Level Match" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GHL All Sources (Booked)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +51,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -76,8 +93,28 @@
         <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00538135"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -99,11 +136,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +201,51 @@
     <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -749,6 +875,763 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PatchitUP of Charlotte — Recommendation Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Now self-funding: optimize for COST PER SOLD ESTIMATE, not lead volume. 'Sold estimate' = GHL won opportunity (quoted work, not collected revenue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Current burn rate (3 paid channels)</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>~$7,340 / month  →  ~17 sold estimates / month  (drained the $15K bundle in ~2 months)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cost / Sold Estimate</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Monthly Run-Rate (as spent)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Angi Subscription</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>$230</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>$980 (fixed)</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>BEST VALUE</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Keep — consider upgrading tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Angi Pay-Per-Lead</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>$417</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>~$1,584</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Efficient</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Keep, but filter by ZIP &amp; category</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Thumbtack</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>$514</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>~$4,780 (63% of spend)</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Over-weighted &amp; costly</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Cut to ~35-40% of budget; fix speed-to-lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Yelp / GLSA / Google PPC</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Unknown (near-zero output)</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Underperforming</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Pause &amp; pull billing before renewing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Website / Referral / Power Partner</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>~$0</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>~$0</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Highest close rate (46-100%)</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Invest time — durable, free pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Spend guardrails</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>1) Keep blended cost-per-sold-estimate UNDER ~15% of your average job value (median sold estimate here was only ~$549 — plug in your real avg ticket).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>2) Target 8-12% of revenue on lead-gen/marketing once booked revenue is known.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>3) Never buy more leads than the crew can service well — match budget to capacity.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A14:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Budget Options — pick by crew capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Expected sold estimates are run-rate estimates at current conversion; the 15-min response rule + filtering should improve them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Option A — Profit-first  (~$2,500/mo)</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="25" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Monthly $</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Expected Sold Est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Angi Subscription</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>980</v>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>~4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Angi Pay-Per-Lead (filtered)</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>800</v>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Thumbtack (tight cap, fast response)</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>700</v>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>~1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Yelp / GLSA / Google</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="n">
+        <v>2480</v>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>~7-8 / mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Option B — Balanced growth  (~$3,800/mo)   ⭐ RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Monthly $</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Expected Sold Est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Angi Subscription</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="n">
+        <v>980</v>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>~4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Angi Pay-Per-Lead (filtered by ZIP/category)</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>~3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Thumbtack (capped, &lt;15-min response)</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>~3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Yelp / GLSA / Google</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>pending review</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="n">
+        <v>3780</v>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>~10-11 / mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Option C — Max volume  (~$5,500/mo)</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="25" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Monthly $</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Expected Sold Est.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Angi Subscription (upgrade)</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n">
+        <v>980</v>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>~4-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Angi Pay-Per-Lead</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>~5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Thumbtack</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>~5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Test Yelp OR Google LSA (measured)</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n">
+        <v>500</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B26" s="34" t="n">
+        <v>5980</v>
+      </c>
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>~14-15 / mo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Action Plan — no-cost fixes + 90-day rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Do these first (free — they raise every channel's return)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>15-minute response rule</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Booked Thumbtack leads were answered in ~144 min; dead leads sat ~752 min (5x slower). Speed is free conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="36" t="inlineStr">
+        <is>
+          <t>Filter Angi &amp; Thumbtack</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Cap by ZIP (stop paying for SC/out-of-area) and category (drop low-value jobs). Dispute spam/out-of-area for refunds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Turn on referral flywheel</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Referrals &amp; power partners closed at 67-100%. Simple 'ask + small reward' + a few HVAC/restoration partners beat any paid channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>Pull Yelp/GLSA/Google billing</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Combined 5 booked / 1 won across the whole book. Get cost data before renewing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>90-day rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Days 1-30</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Move to Option B. Implement 15-min SLA + ZIP/category filters. Pause Yelp/GLSA/Google and pull their reports.</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Days 31-60</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Launch referral + power-partner program. Re-measure cost-per-sold-estimate; shift dollars from Thumbtack to the cheapest Angi product that month.</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Days 61-90</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Decide on Yelp/Google from the cost data. Scale toward Option C ONLY if crew capacity &amp; close rate hold.</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14420,7 +15303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>